<commit_message>
docs : test_evaluation , streamlit install
</commit_message>
<xml_diff>
--- a/volume/test_evaluation.xlsx
+++ b/volume/test_evaluation.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wjddn\Documents\taejung\volume\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f2bf512180cde759/바탕 화면/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{129A8BDD-009A-4840-B9EA-648B046EC5BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1EC385A3-B78C-4086-AF4D-B898885D5AB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="18576" windowHeight="12336" xr2:uid="{324394C1-CEC6-41A5-904B-4EC153A0C5BB}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="19200" windowHeight="11170" xr2:uid="{324394C1-CEC6-41A5-904B-4EC153A0C5BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="43">
   <si>
     <t>Question</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -147,6 +148,60 @@
   </si>
   <si>
     <t>특별한 경우에 재입학이 허용되는 경우는 어떤 경우야?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GS25 위치 알려줘</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GS25 연세플라자 전화번호 알려줘</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>대학교회에 대해 소개해줘</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>재입학 지원 자격 알려줘</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>복학 신청 기간이 어떻게 돼?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>연세플라자 1층에 있는 시설은 어떤게 있어?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>스포츠 시설을 이용할 수 있는 시설은 어디야?</t>
+  </si>
+  <si>
+    <t>카드 발급 받으려면 어디로 가야 돼?</t>
+  </si>
+  <si>
+    <t>건강 관련된 시설은 어떤게 있어?</t>
+  </si>
+  <si>
+    <t>빨래 하려면 어디로 가야 돼?</t>
+  </si>
+  <si>
+    <t>책 사려면 어디로 가야 돼?</t>
+  </si>
+  <si>
+    <t>음식 파는 시설 알려줘</t>
+  </si>
+  <si>
+    <t>버스를 이용하고 싶어</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>서점, GS25 편의점만 답변함 (연세POD센터, 빨래방, 안경점, 구두열쇠점, 우리은행, 우편취급국 X)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BnC 치킨·피자, 학생식당를 답변함(푸드코트는 답변에 없음)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -212,6 +267,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -532,13 +591,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5D7BCB5-E0EB-4092-BE5F-844E24E0B872}">
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="89.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.3984375" customWidth="1"/>
+    <col min="1" max="1" width="89.4140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.4140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -555,7 +614,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -566,7 +625,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -577,7 +636,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -588,7 +647,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -599,7 +658,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -610,7 +669,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -621,7 +680,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -632,7 +691,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -643,7 +702,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -654,7 +713,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -665,7 +724,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -676,7 +735,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -687,7 +746,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -698,7 +757,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -709,7 +768,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -720,7 +779,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -731,7 +790,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -742,7 +801,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>14</v>
       </c>
@@ -753,7 +812,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>15</v>
       </c>
@@ -764,7 +823,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -773,6 +832,188 @@
       </c>
       <c r="F21" t="s">
         <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD7AAFA6-B65C-4639-AC5B-B231E640E671}">
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="67.9140625" customWidth="1"/>
+    <col min="2" max="2" width="12.08203125" customWidth="1"/>
+    <col min="7" max="7" width="116.4140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" t="s">
+        <v>22</v>
+      </c>
+      <c r="G13" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>